<commit_message>
TAREFA 07 parcialmente concluída
</commit_message>
<xml_diff>
--- a/Avancado/07 - ÍNDICE e CORRESP.xlsx
+++ b/Avancado/07 - ÍNDICE e CORRESP.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4727BEC0-C478-43C3-92C5-5EB45FD43115}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +24,89 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+  <si>
+    <t>Controlador de Entrada e Saída</t>
+  </si>
+  <si>
+    <t>Cargo</t>
+  </si>
+  <si>
+    <t>Controlador de Pragas</t>
+  </si>
+  <si>
+    <t>Cozinheiro Geral</t>
+  </si>
+  <si>
+    <t>Abatedor</t>
+  </si>
+  <si>
+    <t>Acabador de Calçados</t>
+  </si>
+  <si>
+    <t>Açougueiro</t>
+  </si>
+  <si>
+    <t>Acrobata</t>
+  </si>
+  <si>
+    <t>Adestrador de Animais</t>
+  </si>
+  <si>
+    <t>Administrador</t>
+  </si>
+  <si>
+    <t>Administrador de Edifícios</t>
+  </si>
+  <si>
+    <t>Administrador de Redes</t>
+  </si>
+  <si>
+    <t>Advogado</t>
+  </si>
+  <si>
+    <t>Advogado (Direito Cívil)</t>
+  </si>
+  <si>
+    <t>Compensador de Banco</t>
+  </si>
+  <si>
+    <t>Compositor</t>
+  </si>
+  <si>
+    <t>Comprador</t>
+  </si>
+  <si>
+    <t>Consultor Jurídico</t>
+  </si>
+  <si>
+    <t>Contador</t>
+  </si>
+  <si>
+    <t>Continuo</t>
+  </si>
+  <si>
+    <t>Condutor de Veículo a Pedais</t>
+  </si>
+  <si>
+    <t>Piso Salarial</t>
+  </si>
+  <si>
+    <t>CBO</t>
+  </si>
+  <si>
+    <t>Salário Aprendiz</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="&quot;CBO &quot;0000&quot;-&quot;00"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +114,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -45,12 +145,218 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +636,424 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="10"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="15"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1011.71</v>
+      </c>
+      <c r="C2" s="5">
+        <v>848505</v>
+      </c>
+      <c r="D2" s="4">
+        <v>495.23</v>
+      </c>
+      <c r="E2" s="10"/>
+      <c r="F2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="8">
+        <v>513205</v>
+      </c>
+      <c r="H2" s="16"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1013.68</v>
+      </c>
+      <c r="C3" s="5">
+        <v>764305</v>
+      </c>
+      <c r="D3" s="4">
+        <v>389.49</v>
+      </c>
+      <c r="E3" s="10"/>
+      <c r="F3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="str">
+        <f>INDEX($A$2:$D$21,MATCH($G$2,$C$2:$C$21,0),MATCH($F3,$A$1:$D$1,0))</f>
+        <v>Cozinheiro Geral</v>
+      </c>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1064.21</v>
+      </c>
+      <c r="C4" s="5">
+        <v>848510</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="4">
+        <f>INDEX($A$2:$D$21,MATCH($G$2,$C$2:$C$21,0),MATCH($F4,$A$1:$D$1,0))</f>
+        <v>1008.69</v>
+      </c>
+      <c r="H4" s="16"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="19"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1462.06</v>
+      </c>
+      <c r="C5" s="5">
+        <v>376205</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="4">
+        <f>INDEX($A$2:$D$21,MATCH($G$2,$C$2:$C$21,0),MATCH($F5,$A$1:$D$1,0))</f>
+        <v>867.02</v>
+      </c>
+      <c r="H5" s="16"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1301.1300000000001</v>
+      </c>
+      <c r="C6" s="5">
+        <v>623005</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="15"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4">
+        <v>3294.51</v>
+      </c>
+      <c r="C7" s="5">
+        <v>252105</v>
+      </c>
+      <c r="D7" s="4">
+        <v>635.88</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="15"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1785.7</v>
+      </c>
+      <c r="C8" s="5">
+        <v>510110</v>
+      </c>
+      <c r="D8" s="4">
+        <v>484</v>
+      </c>
+      <c r="E8" s="10"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4">
+        <v>3213.72</v>
+      </c>
+      <c r="C9" s="5">
+        <v>212310</v>
+      </c>
+      <c r="D9" s="4">
+        <v>522.4</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="15"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4">
+        <v>3169.51</v>
+      </c>
+      <c r="C10" s="5">
+        <v>241005</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="10"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="15"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4">
+        <v>3368.31</v>
+      </c>
+      <c r="C11" s="5">
+        <v>241015</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4">
+        <v>954</v>
+      </c>
+      <c r="C12" s="5">
+        <v>413215</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="15"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4">
+        <v>4800</v>
+      </c>
+      <c r="C13" s="5">
+        <v>262605</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="15"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4">
+        <v>2591.27</v>
+      </c>
+      <c r="C14" s="5">
+        <v>354205</v>
+      </c>
+      <c r="D14" s="4">
+        <v>970</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="15"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4">
+        <v>954</v>
+      </c>
+      <c r="C15" s="5">
+        <v>782820</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="15"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="4">
+        <v>3479.43</v>
+      </c>
+      <c r="C16" s="5">
+        <v>241040</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="4">
+        <v>3297.34</v>
+      </c>
+      <c r="C17" s="5">
+        <v>252210</v>
+      </c>
+      <c r="D17" s="4">
+        <v>676</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="15"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="4">
+        <v>954</v>
+      </c>
+      <c r="C18" s="5">
+        <v>412205</v>
+      </c>
+      <c r="D18" s="4">
+        <v>675.1</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="15"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="4">
+        <v>1173.74</v>
+      </c>
+      <c r="C19" s="5">
+        <v>391115</v>
+      </c>
+      <c r="D19" s="4">
+        <v>690.85</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="15"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1044.71</v>
+      </c>
+      <c r="C20" s="5">
+        <v>519910</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="10"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="15"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="4">
+        <v>1008.69</v>
+      </c>
+      <c r="C21" s="5">
+        <v>513205</v>
+      </c>
+      <c r="D21" s="4">
+        <v>867.02</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="17"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{599EEEFA-8E48-4916-AB98-2E1B06F9FA06}">
+      <formula1>$C$2:$C$21</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>